<commit_message>
Update data - 2025-08-05 12:50:02
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,77 +468,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Allie George</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bev</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ab</t>
+          <t>vs Palmerias</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>vs Palmerias</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Kayla Fischer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -569,7 +565,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kayla Fischer</t>
+          <t>Sarah Weber</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -600,7 +596,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sarah Weber</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -631,7 +627,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -662,7 +658,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -693,38 +689,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>vs Lexington &amp; São Paolo</t>
+        </is>
+      </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington &amp; São Paolo</t>
+          <t>vs Lexington</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,19 +782,15 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>vs Lexington</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -825,7 +821,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -856,7 +852,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -887,7 +883,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -918,7 +914,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -949,62 +945,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Bev &amp; Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ella Hase</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Bev &amp; Mitch</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-08-05 13:02:37
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,67 +468,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Allie George</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-08-05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Bev</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>vs Palmerias</t>
+          <t>abc</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>vs Palmerias</t>
+        </is>
+      </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -689,42 +693,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>vs Lexington &amp; São Paolo</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington</t>
+          <t>vs Lexington &amp; São Paolo</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,15 +782,19 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>vs Lexington</t>
+        </is>
+      </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -821,7 +825,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -852,7 +856,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -883,7 +887,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -914,7 +918,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -945,31 +949,62 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bev &amp; Mitch</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ella Hase</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bev &amp; Mitch</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-08-05 13:15:19
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,77 +468,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Allie George</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bev</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>vs Palmerias</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Kayla Fischer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>vs Palmerias</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kayla Fischer</t>
+          <t>Sarah Weber</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -569,7 +565,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sarah Weber</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -600,7 +596,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -631,7 +627,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -662,7 +658,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -693,38 +689,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>vs Lexington &amp; São Paolo</t>
+        </is>
+      </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington &amp; São Paolo</t>
+          <t>vs Lexington</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,19 +782,15 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>vs Lexington</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -825,7 +821,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -856,7 +852,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -887,7 +883,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -918,7 +914,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -949,62 +945,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Bev &amp; Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ella Hase</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Bev &amp; Mitch</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-08-13 20:57:18
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,67 +468,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Ary Borges</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>1v1 Defending</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-08-13</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>vs Palmerias</t>
+          <t>Pre Match - MD 17</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kayla Fischer</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>vs Palmerias</t>
+        </is>
+      </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -689,42 +693,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Kayla Fischer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>vs Lexington &amp; São Paolo</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington</t>
+          <t>vs Lexington &amp; São Paolo</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,15 +782,19 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>vs Lexington</t>
+        </is>
+      </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -821,7 +825,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -852,7 +856,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -883,7 +887,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -914,7 +918,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -945,31 +949,62 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bev &amp; Mitch</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ella Hase</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bev &amp; Mitch</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-08-13 20:57:37
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,77 +468,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ary Borges</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1v1 Defending</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-08-13</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pre Match - MD 17</t>
+          <t>vs Palmerias</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Sarah Weber</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>vs Palmerias</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sarah Weber</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -569,7 +565,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -600,7 +596,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -631,7 +627,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -662,7 +658,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Kayla Fischer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -693,38 +689,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kayla Fischer</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>vs Lexington &amp; São Paolo</t>
+        </is>
+      </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington &amp; São Paolo</t>
+          <t>vs Lexington</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,19 +782,15 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>vs Lexington</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -825,7 +821,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -856,7 +852,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -887,7 +883,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -918,7 +914,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -949,62 +945,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Bev &amp; Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ella Hase</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Bev &amp; Mitch</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-09-02 14:55:43
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,67 +468,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Courtney Petersen</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>vs Palmerias</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sarah Weber</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>vs Palmerias</t>
+        </is>
+      </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -689,42 +689,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Sarah Weber</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>vs Lexington &amp; São Paolo</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -739,7 +735,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -749,32 +745,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington</t>
+          <t>vs Lexington &amp; São Paolo</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -782,15 +778,19 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>vs Lexington</t>
+        </is>
+      </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -914,7 +914,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -945,31 +945,62 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bev &amp; Mitch</t>
+          <t>Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ella Hase</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bev &amp; Mitch</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data - 2025-09-02 15:00:59
</commit_message>
<xml_diff>
--- a/MitchIDPs.xlsx
+++ b/MitchIDPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,73 +468,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Courtney Petersen</t>
+          <t>Ellie Jean</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-09-02</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>vs Palmerias</t>
+        </is>
+      </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ellie Jean</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Combined</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-07-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mitch</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>vs Palmerias</t>
-        </is>
-      </c>
+          <t>Bev</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -627,7 +627,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Kayla Fischer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -658,7 +658,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kayla Fischer</t>
+          <t>Sarah Weber</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -689,38 +689,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sarah Weber</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combined</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-07-23</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bev</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Mitch</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>vs Lexington &amp; São Paolo</t>
+        </is>
+      </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -735,7 +739,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-07-23</t>
+          <t>2025-07-18</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -745,32 +749,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>vs Lexington &amp; São Paolo</t>
+          <t>vs Lexington</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ella Hase</t>
+          <t>Bethany Balcer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Group</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Finishing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-07-18</t>
+          <t>2025-07-15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -778,19 +782,15 @@
           <t>Mitch</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>vs Lexington</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bethany Balcer</t>
+          <t>Katie O'Kane</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Katie O'Kane</t>
+          <t>Savannah DeMelo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Savannah DeMelo</t>
+          <t>Uchenna Kanu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uchenna Kanu</t>
+          <t>Marisa DiGrande</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -914,7 +914,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marisa DiGrande</t>
+          <t>Jordan Baggett</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -945,62 +945,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jordan Baggett</t>
+          <t>Ella Hase</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Finishing</t>
+          <t>Overall</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-07-15</t>
+          <t>2025-07-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mitch</t>
+          <t>Bev &amp; Mitch</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ella Hase</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Bev &amp; Mitch</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>